<commit_message>
feat: feita correção nas formas de pagamemto
</commit_message>
<xml_diff>
--- a/data/processed/Cassio_Tratada.xlsx
+++ b/data/processed/Cassio_Tratada.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Logan\barbearia-dados-pandas\data\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0702795F-CE2D-4FA6-BDC2-83DB071F7C0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDEF5063-4AB2-4B32-9EB6-0C06315556C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -6840,7 +6840,7 @@
         <v>31</v>
       </c>
       <c r="K126" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="O126">
         <v>80</v>

</xml_diff>